<commit_message>
Add organization map geocoding debug logging and update statistics
</commit_message>
<xml_diff>
--- a/mts/KGR-PEOPLE.xlsx
+++ b/mts/KGR-PEOPLE.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1010">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1236" count="1236">
   <si>
     <t>This document was exported from Numbers.  Each table was converted to an Excel worksheet. All other objects on each Numbers sheet were placed on separate worksheets. Please be aware that formula calculations may differ in Excel.</t>
   </si>
@@ -2692,12 +2692,12 @@
     <t>Pinheiro</t>
   </si>
   <si>
+    <t>https://pmsr.net/ont/ORG174547867570630937</t>
+  </si>
+  <si>
     <t>mailto:paulo.pinheiro@ipiaget.pt</t>
   </si>
   <si>
-    <t>https://pmsr.net/ont/ORG174547867570630937</t>
-  </si>
-  <si>
     <t>https://pmsr.net/ont/Person_002</t>
   </si>
   <si>
@@ -2710,12 +2710,12 @@
     <t>Moreira</t>
   </si>
   <si>
+    <t>https://pmsr.net/ont/ORG174547867570665413</t>
+  </si>
+  <si>
     <t>mailto:luis.moreira@ipiaget.pt</t>
   </si>
   <si>
-    <t>https://pmsr.net/ont/ORG174547867570665413</t>
-  </si>
-  <si>
     <t>https://pmsr.net/ont/Person_003</t>
   </si>
   <si>
@@ -2800,12 +2800,12 @@
     <t>Gagulic</t>
   </si>
   <si>
+    <t>https://pmsr.net/ont/ORG174547834502854654</t>
+  </si>
+  <si>
     <t>mailto:sandra.gagulic@ipiaget.pt</t>
   </si>
   <si>
-    <t>https://pmsr.net/ont/ORG174547834502854654</t>
-  </si>
-  <si>
     <t>https://pmsr.net/ont/Person_009</t>
   </si>
   <si>
@@ -3050,6 +3050,684 @@
   </si>
   <si>
     <t>schema:postalCode</t>
+  </si>
+  <si>
+    <t>hasco:userName</t>
+  </si>
+  <si>
+    <t>hasco:userEmail</t>
+  </si>
+  <si>
+    <t>hasco:userID</t>
+  </si>
+  <si>
+    <t>Amandine Azevedo</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Amandine</t>
+  </si>
+  <si>
+    <t>Azevedo</t>
+  </si>
+  <si>
+    <t>https://pmsr.net/ont/ORG174547834502816317</t>
+  </si>
+  <si>
+    <t>amandine.azevedo@isave.pt</t>
+  </si>
+  <si>
+    <t>AmandineAzevedo</t>
+  </si>
+  <si>
+    <t>Ana Caldeira</t>
+  </si>
+  <si>
+    <t>69</t>
+  </si>
+  <si>
+    <t>Ana</t>
+  </si>
+  <si>
+    <t>Caldeira</t>
+  </si>
+  <si>
+    <t>https://pmsr.net/ont/ORG174547834502848251</t>
+  </si>
+  <si>
+    <t>ana.caldeira@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>AnaCaldeira</t>
+  </si>
+  <si>
+    <t>Andreia Goncalves</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>Andreia</t>
+  </si>
+  <si>
+    <t>Goncalves</t>
+  </si>
+  <si>
+    <t>https://pmsr.net/ont/ORG_PMSR</t>
+  </si>
+  <si>
+    <t>andreiagoncalves@pmsr.net</t>
+  </si>
+  <si>
+    <t>AndreiaGoncalves</t>
+  </si>
+  <si>
+    <t>Andreina Tavares</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>Andreina</t>
+  </si>
+  <si>
+    <t>Tavares</t>
+  </si>
+  <si>
+    <t>andreina.tavares@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>AndreinaTavares</t>
+  </si>
+  <si>
+    <t>Andre Leao</t>
+  </si>
+  <si>
+    <t>74</t>
+  </si>
+  <si>
+    <t>Andre</t>
+  </si>
+  <si>
+    <t>Leao</t>
+  </si>
+  <si>
+    <t>andre.leao@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>AndreLeao</t>
+  </si>
+  <si>
+    <t>Andre Novo</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>Novo</t>
+  </si>
+  <si>
+    <t>https://pmsr.net/ont/ORG174547834502882527</t>
+  </si>
+  <si>
+    <t>andre@ipb.pt</t>
+  </si>
+  <si>
+    <t>AndreNovo</t>
+  </si>
+  <si>
+    <t>Andre Rodrigues</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>Rodrigues</t>
+  </si>
+  <si>
+    <t>andre.rodrigues@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>AndreRodrigues</t>
+  </si>
+  <si>
+    <t>Antonio Ferreira</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>Antonio</t>
+  </si>
+  <si>
+    <t>https://pmsr.net/ont/ORG174547834502817893</t>
+  </si>
+  <si>
+    <t>antonio.ferreira@essnortecvp.pt</t>
+  </si>
+  <si>
+    <t>AntonioFerreira</t>
+  </si>
+  <si>
+    <t>Carlos Tavares</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>Carlos</t>
+  </si>
+  <si>
+    <t>carlos.tavares@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>CarlosTavares</t>
+  </si>
+  <si>
+    <t>Catarina Valente</t>
+  </si>
+  <si>
+    <t>77</t>
+  </si>
+  <si>
+    <t>Catarina</t>
+  </si>
+  <si>
+    <t>catarina.valente@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>CatarinaValente</t>
+  </si>
+  <si>
+    <t>Daniel Martins</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>Daniel</t>
+  </si>
+  <si>
+    <t>Martins</t>
+  </si>
+  <si>
+    <t>daniel.martins@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>DanielMartins</t>
+  </si>
+  <si>
+    <t>Ines Bento</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>Ines</t>
+  </si>
+  <si>
+    <t>Bento</t>
+  </si>
+  <si>
+    <t>https://pmsr.net/ont/ORG174547834502865973</t>
+  </si>
+  <si>
+    <t>ibento@esscvp.eu</t>
+  </si>
+  <si>
+    <t>InesBento</t>
+  </si>
+  <si>
+    <t>Isabel Alves</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>Isabel</t>
+  </si>
+  <si>
+    <t>Alves</t>
+  </si>
+  <si>
+    <t>isabel.alves@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>IsabelAlves</t>
+  </si>
+  <si>
+    <t>67</t>
+  </si>
+  <si>
+    <t>joana.pinto@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>JoanaPinto</t>
+  </si>
+  <si>
+    <t>Joana Silva</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>Silva</t>
+  </si>
+  <si>
+    <t>joana.paula@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>JoanaSilva</t>
+  </si>
+  <si>
+    <t>72</t>
+  </si>
+  <si>
+    <t>joana.teixeira@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>JoanaTeixeira</t>
+  </si>
+  <si>
+    <t>Joao Amado</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>Joao</t>
+  </si>
+  <si>
+    <t>Amado</t>
+  </si>
+  <si>
+    <t>https://pmsr.net/ont/ORG174547834502838939</t>
+  </si>
+  <si>
+    <t>jamado@ucp.pt</t>
+  </si>
+  <si>
+    <t>JoaoAmado</t>
+  </si>
+  <si>
+    <t>Joao Grade</t>
+  </si>
+  <si>
+    <t>62</t>
+  </si>
+  <si>
+    <t>joao.grade@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>JoaoGrade</t>
+  </si>
+  <si>
+    <t>Joao Rosa</t>
+  </si>
+  <si>
+    <t>53</t>
+  </si>
+  <si>
+    <t>Rosa</t>
+  </si>
+  <si>
+    <t>https://pmsr.net/ont/ORG174547867570660682</t>
+  </si>
+  <si>
+    <t>j.rosa@ess.ipvc.pt</t>
+  </si>
+  <si>
+    <t>JoaoRosa</t>
+  </si>
+  <si>
+    <t>Joao Simoes</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>Simoes</t>
+  </si>
+  <si>
+    <t>https://pmsr.net/ont/ORG174547834502849898</t>
+  </si>
+  <si>
+    <t>jflindo@ua.pt</t>
+  </si>
+  <si>
+    <t>JoaoSimoes</t>
+  </si>
+  <si>
+    <t>Joaquim Papanca</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>Joaquim</t>
+  </si>
+  <si>
+    <t>Papanca</t>
+  </si>
+  <si>
+    <t>joaquim.papanca@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>JoaquimPapanca</t>
+  </si>
+  <si>
+    <t>Jose Alvarelhao</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>Jose</t>
+  </si>
+  <si>
+    <t>Alvarelhao</t>
+  </si>
+  <si>
+    <t>jalvarelhao@ua.pt</t>
+  </si>
+  <si>
+    <t>JoseAlvarelhao</t>
+  </si>
+  <si>
+    <t>Karla Bandeira</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>Karla</t>
+  </si>
+  <si>
+    <t>Bandeira</t>
+  </si>
+  <si>
+    <t>https://pmsr.net/ont/ORG_EXTERNAL_GRAXIOM</t>
+  </si>
+  <si>
+    <t>karla@graxiom.com</t>
+  </si>
+  <si>
+    <t>KarlaBandeira</t>
+  </si>
+  <si>
+    <t>Leila Sales</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>Leila</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>lsales@esscvp.eu</t>
+  </si>
+  <si>
+    <t>LeilaSales</t>
+  </si>
+  <si>
+    <t>Liliana Mota Liliana Mota</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>Liliana</t>
+  </si>
+  <si>
+    <t>Mota Liliana Mota</t>
+  </si>
+  <si>
+    <t>liliana.mota@essnortecvp.pt</t>
+  </si>
+  <si>
+    <t>LilianaMotaLilianaMota</t>
+  </si>
+  <si>
+    <t>Lucia Pereira</t>
+  </si>
+  <si>
+    <t>63</t>
+  </si>
+  <si>
+    <t>Lucia</t>
+  </si>
+  <si>
+    <t>lucia.pereira@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>LuciaPereira</t>
+  </si>
+  <si>
+    <t>Luis Graca</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>Graca</t>
+  </si>
+  <si>
+    <t>luisgraca@ess.ipvc.pt</t>
+  </si>
+  <si>
+    <t>LuisGraca</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>luis.moreira@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>LuisMoreira</t>
+  </si>
+  <si>
+    <t>66</t>
+  </si>
+  <si>
+    <t>margarida.v.ferreira@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>MargaridaFerreira</t>
+  </si>
+  <si>
+    <t>Mario Rodrigues</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>Mario</t>
+  </si>
+  <si>
+    <t>mmpr@ua.pt</t>
+  </si>
+  <si>
+    <t>MarioRodrigues</t>
+  </si>
+  <si>
+    <t>Maria Sousa</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>Maria</t>
+  </si>
+  <si>
+    <t>mariajoao.sousa@isave.pt</t>
+  </si>
+  <si>
+    <t>MariaSousa</t>
+  </si>
+  <si>
+    <t>Natanael Quintino</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>Natanael</t>
+  </si>
+  <si>
+    <t>Quintino</t>
+  </si>
+  <si>
+    <t>natanael.quintino@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>NatanaelQuintino</t>
+  </si>
+  <si>
+    <t>Nelson Sousa</t>
+  </si>
+  <si>
+    <t>64</t>
+  </si>
+  <si>
+    <t>Nelson</t>
+  </si>
+  <si>
+    <t>nelson.sousa@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>NelsonSousa</t>
+  </si>
+  <si>
+    <t>Nuno Simoes</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>Nuno</t>
+  </si>
+  <si>
+    <t>nunosimoes@graxiom.com</t>
+  </si>
+  <si>
+    <t>NunoSimoes</t>
+  </si>
+  <si>
+    <t>Paula Borges</t>
+  </si>
+  <si>
+    <t>71</t>
+  </si>
+  <si>
+    <t>Paula</t>
+  </si>
+  <si>
+    <t>paula.borges@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>PaulaBorges</t>
+  </si>
+  <si>
+    <t>Paulo Alves</t>
+  </si>
+  <si>
+    <t>34</t>
+  </si>
+  <si>
+    <t>pjalves@ucp.pt</t>
+  </si>
+  <si>
+    <t>PauloAlves</t>
+  </si>
+  <si>
+    <t>Paulo Azevedo</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>paulo.azevedo@essnortecvp.pt</t>
+  </si>
+  <si>
+    <t>PauloAzevedo</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>pp3223@gmail.com</t>
+  </si>
+  <si>
+    <t>PauloPinheiro</t>
+  </si>
+  <si>
+    <t>Pedro Araujo</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>Pedro</t>
+  </si>
+  <si>
+    <t>Araujo</t>
+  </si>
+  <si>
+    <t>pedroaraujo@ess.ipvc.pt</t>
+  </si>
+  <si>
+    <t>PedroAraujo</t>
+  </si>
+  <si>
+    <t>Pedro Lopes</t>
+  </si>
+  <si>
+    <t>73</t>
+  </si>
+  <si>
+    <t>pedro.lopes@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>PedroLopes</t>
+  </si>
+  <si>
+    <t>70</t>
+  </si>
+  <si>
+    <t>sandra.gagulic@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>SandraGagulic</t>
+  </si>
+  <si>
+    <t>Tiago Moreira</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Tiago</t>
+  </si>
+  <si>
+    <t>tiagomoreira@graxiom.com</t>
+  </si>
+  <si>
+    <t>TiagoMoreira</t>
+  </si>
+  <si>
+    <t>65</t>
+  </si>
+  <si>
+    <t>veronica.abreu@ipiaget.pt</t>
+  </si>
+  <si>
+    <t>VeronicaAbreu</t>
   </si>
 </sst>
 </file>
@@ -8794,22 +9472,22 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:L24"/>
   <sheetFormatPr defaultColWidth="10.6667" defaultRowHeight="12.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="9.5" style="14" customWidth="1"/>
     <col min="2" max="2" width="21.3516" style="14" customWidth="1"/>
-    <col min="3" max="3" width="12.1719" style="14" customWidth="1"/>
+    <col min="3" max="3" width="38.5547" style="14" customWidth="1"/>
     <col min="4" max="4" width="20" style="14" customWidth="1"/>
     <col min="5" max="5" width="10.5" style="14" customWidth="1"/>
     <col min="6" max="6" width="19.6719" style="14" customWidth="1"/>
     <col min="7" max="7" width="20.5" style="14" customWidth="1"/>
-    <col min="8" max="8" width="42.8047" style="14" customWidth="1"/>
-    <col min="9" max="9" width="36.1719" style="14" customWidth="1"/>
-    <col min="10" max="10" width="20.1719" style="14" customWidth="1"/>
-    <col min="11" max="11" width="30.1719" style="14" customWidth="1"/>
-    <col min="12" max="12" width="17.5" style="14" customWidth="1"/>
+    <col min="8" max="8" width="20.1719" style="14" customWidth="1"/>
+    <col min="9" max="9" width="19.6719" style="14" customWidth="1"/>
+    <col min="10" max="10" width="43.9609" style="14" customWidth="1"/>
+    <col min="11" max="11" width="38.8281" style="14" customWidth="1"/>
+    <col min="12" max="12" width="31.8594" style="14" customWidth="1"/>
     <col min="13" max="16384" width="10.6719" style="14" customWidth="1"/>
   </cols>
   <sheetData>
@@ -8836,19 +9514,28 @@
         <v>883</v>
       </c>
       <c r="H1" t="s" s="7">
+        <v>43</v>
+      </c>
+      <c r="I1" t="s" s="7">
+        <v>44</v>
+      </c>
+      <c r="J1" t="s" s="7">
+        <v>42</v>
+      </c>
+      <c r="K1" t="s" s="7">
+        <v>884</v>
+      </c>
+      <c r="L1" t="s" s="7">
         <v>50</v>
       </c>
-      <c r="I1" t="s" s="7">
-        <v>884</v>
-      </c>
-      <c r="J1" t="s" s="7">
-        <v>43</v>
-      </c>
-      <c r="K1" t="s" s="7">
-        <v>44</v>
-      </c>
-      <c r="L1" t="s" s="7">
-        <v>42</v>
+      <c r="M1" t="s">
+        <v>1010</v>
+      </c>
+      <c r="N1" t="s">
+        <v>1011</v>
+      </c>
+      <c r="O1" t="s">
+        <v>1012</v>
       </c>
     </row>
     <row r="2" ht="13.65" customHeight="1">
@@ -8871,15 +9558,17 @@
       <c r="G2" t="s" s="7">
         <v>889</v>
       </c>
-      <c r="H2" t="s" s="7">
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" t="s" s="7">
+        <v>887</v>
+      </c>
+      <c r="K2" t="s" s="7">
         <v>890</v>
       </c>
-      <c r="I2" t="s" s="7">
+      <c r="L2" t="s" s="7">
         <v>891</v>
       </c>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
     </row>
     <row r="3" ht="13.65" customHeight="1">
       <c r="A3" t="s" s="7">
@@ -8901,15 +9590,17 @@
       <c r="G3" t="s" s="7">
         <v>895</v>
       </c>
-      <c r="H3" t="s" s="7">
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" t="s" s="7">
+        <v>893</v>
+      </c>
+      <c r="K3" t="s" s="7">
         <v>896</v>
       </c>
-      <c r="I3" t="s" s="7">
+      <c r="L3" t="s" s="7">
         <v>897</v>
       </c>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-      <c r="L3" s="8"/>
     </row>
     <row r="4" ht="13.65" customHeight="1">
       <c r="A4" t="s" s="7">
@@ -8931,15 +9622,17 @@
       <c r="G4" t="s" s="7">
         <v>901</v>
       </c>
-      <c r="H4" t="s" s="7">
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+      <c r="J4" t="s" s="7">
+        <v>899</v>
+      </c>
+      <c r="K4" t="s" s="7">
+        <v>896</v>
+      </c>
+      <c r="L4" t="s" s="7">
         <v>902</v>
       </c>
-      <c r="I4" t="s" s="7">
-        <v>897</v>
-      </c>
-      <c r="J4" s="8"/>
-      <c r="K4" s="8"/>
-      <c r="L4" s="8"/>
     </row>
     <row r="5" ht="13.65" customHeight="1">
       <c r="A5" t="s" s="7">
@@ -8961,15 +9654,17 @@
       <c r="G5" t="s" s="7">
         <v>905</v>
       </c>
-      <c r="H5" t="s" s="7">
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
+      <c r="J5" t="s" s="7">
+        <v>904</v>
+      </c>
+      <c r="K5" t="s" s="7">
+        <v>896</v>
+      </c>
+      <c r="L5" t="s" s="7">
         <v>906</v>
       </c>
-      <c r="I5" t="s" s="7">
-        <v>897</v>
-      </c>
-      <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
-      <c r="L5" s="8"/>
     </row>
     <row r="6" ht="13.65" customHeight="1">
       <c r="A6" t="s" s="7">
@@ -8991,15 +9686,17 @@
       <c r="G6" t="s" s="7">
         <v>910</v>
       </c>
-      <c r="H6" t="s" s="7">
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" t="s" s="7">
+        <v>908</v>
+      </c>
+      <c r="K6" t="s" s="7">
+        <v>896</v>
+      </c>
+      <c r="L6" t="s" s="7">
         <v>911</v>
       </c>
-      <c r="I6" t="s" s="7">
-        <v>897</v>
-      </c>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
-      <c r="L6" s="8"/>
     </row>
     <row r="7" ht="13.65" customHeight="1">
       <c r="A7" t="s" s="7">
@@ -9021,15 +9718,17 @@
       <c r="G7" t="s" s="7">
         <v>915</v>
       </c>
-      <c r="H7" t="s" s="7">
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" t="s" s="7">
+        <v>913</v>
+      </c>
+      <c r="K7" t="s" s="7">
+        <v>896</v>
+      </c>
+      <c r="L7" t="s" s="7">
         <v>916</v>
       </c>
-      <c r="I7" t="s" s="7">
-        <v>897</v>
-      </c>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
-      <c r="L7" s="8"/>
     </row>
     <row r="8" ht="13.65" customHeight="1">
       <c r="A8" t="s" s="7">
@@ -9051,15 +9750,17 @@
       <c r="G8" t="s" s="7">
         <v>920</v>
       </c>
-      <c r="H8" t="s" s="7">
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" t="s" s="7">
+        <v>918</v>
+      </c>
+      <c r="K8" t="s" s="7">
+        <v>896</v>
+      </c>
+      <c r="L8" t="s" s="7">
         <v>921</v>
       </c>
-      <c r="I8" t="s" s="7">
-        <v>897</v>
-      </c>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="8"/>
     </row>
     <row r="9" ht="13.65" customHeight="1">
       <c r="A9" t="s" s="7">
@@ -9081,15 +9782,17 @@
       <c r="G9" t="s" s="7">
         <v>925</v>
       </c>
-      <c r="H9" t="s" s="7">
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" t="s" s="7">
+        <v>923</v>
+      </c>
+      <c r="K9" t="s" s="7">
         <v>926</v>
       </c>
-      <c r="I9" t="s" s="7">
+      <c r="L9" t="s" s="7">
         <v>927</v>
       </c>
-      <c r="J9" s="8"/>
-      <c r="K9" s="8"/>
-      <c r="L9" s="8"/>
     </row>
     <row r="10" ht="13.65" customHeight="1">
       <c r="A10" t="s" s="7">
@@ -9111,15 +9814,17 @@
       <c r="G10" t="s" s="7">
         <v>931</v>
       </c>
-      <c r="H10" t="s" s="7">
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" t="s" s="7">
+        <v>929</v>
+      </c>
+      <c r="K10" t="s" s="7">
+        <v>926</v>
+      </c>
+      <c r="L10" t="s" s="7">
         <v>932</v>
       </c>
-      <c r="I10" t="s" s="7">
-        <v>927</v>
-      </c>
-      <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="8"/>
     </row>
     <row r="11" ht="13.65" customHeight="1">
       <c r="A11" t="s" s="7">
@@ -9141,15 +9846,17 @@
       <c r="G11" t="s" s="7">
         <v>936</v>
       </c>
-      <c r="H11" t="s" s="7">
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" t="s" s="7">
+        <v>934</v>
+      </c>
+      <c r="K11" t="s" s="7">
+        <v>896</v>
+      </c>
+      <c r="L11" t="s" s="7">
         <v>937</v>
       </c>
-      <c r="I11" t="s" s="7">
-        <v>897</v>
-      </c>
-      <c r="J11" s="8"/>
-      <c r="K11" s="8"/>
-      <c r="L11" s="8"/>
     </row>
     <row r="12" ht="13.65" customHeight="1">
       <c r="A12" t="s" s="7">
@@ -9171,15 +9878,17 @@
       <c r="G12" t="s" s="7">
         <v>940</v>
       </c>
-      <c r="H12" t="s" s="7">
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" t="s" s="7">
+        <v>939</v>
+      </c>
+      <c r="K12" t="s" s="7">
+        <v>896</v>
+      </c>
+      <c r="L12" t="s" s="7">
         <v>941</v>
       </c>
-      <c r="I12" t="s" s="7">
-        <v>897</v>
-      </c>
-      <c r="J12" s="8"/>
-      <c r="K12" s="8"/>
-      <c r="L12" s="8"/>
     </row>
     <row r="13" ht="13.65" customHeight="1">
       <c r="A13" t="s" s="7">
@@ -9201,15 +9910,17 @@
       <c r="G13" t="s" s="7">
         <v>945</v>
       </c>
-      <c r="H13" t="s" s="7">
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" t="s" s="7">
+        <v>943</v>
+      </c>
+      <c r="K13" t="s" s="7">
+        <v>896</v>
+      </c>
+      <c r="L13" t="s" s="7">
         <v>946</v>
       </c>
-      <c r="I13" t="s" s="7">
-        <v>897</v>
-      </c>
-      <c r="J13" s="8"/>
-      <c r="K13" s="8"/>
-      <c r="L13" s="8"/>
     </row>
     <row r="14" ht="13.65" customHeight="1">
       <c r="A14" t="s" s="7">
@@ -9231,15 +9942,17 @@
       <c r="G14" t="s" s="7">
         <v>950</v>
       </c>
-      <c r="H14" t="s" s="7">
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" t="s" s="7">
+        <v>948</v>
+      </c>
+      <c r="K14" t="s" s="7">
+        <v>896</v>
+      </c>
+      <c r="L14" t="s" s="7">
         <v>951</v>
       </c>
-      <c r="I14" t="s" s="7">
-        <v>897</v>
-      </c>
-      <c r="J14" s="8"/>
-      <c r="K14" s="8"/>
-      <c r="L14" s="8"/>
     </row>
     <row r="15" ht="13.65" customHeight="1">
       <c r="A15" t="s" s="7">
@@ -9261,15 +9974,17 @@
       <c r="G15" t="s" s="7">
         <v>955</v>
       </c>
-      <c r="H15" t="s" s="7">
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" t="s" s="7">
+        <v>953</v>
+      </c>
+      <c r="K15" t="s" s="7">
+        <v>926</v>
+      </c>
+      <c r="L15" t="s" s="7">
         <v>956</v>
       </c>
-      <c r="I15" t="s" s="7">
-        <v>927</v>
-      </c>
-      <c r="J15" s="8"/>
-      <c r="K15" s="8"/>
-      <c r="L15" s="8"/>
     </row>
     <row r="16" ht="13.65" customHeight="1">
       <c r="A16" t="s" s="7">
@@ -9291,15 +10006,17 @@
       <c r="G16" t="s" s="7">
         <v>960</v>
       </c>
-      <c r="H16" t="s" s="7">
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" t="s" s="7">
+        <v>958</v>
+      </c>
+      <c r="K16" t="s" s="7">
+        <v>926</v>
+      </c>
+      <c r="L16" t="s" s="7">
         <v>961</v>
       </c>
-      <c r="I16" t="s" s="7">
-        <v>927</v>
-      </c>
-      <c r="J16" s="8"/>
-      <c r="K16" s="8"/>
-      <c r="L16" s="8"/>
     </row>
     <row r="17" ht="13.65" customHeight="1">
       <c r="A17" t="s" s="7">
@@ -9321,15 +10038,17 @@
       <c r="G17" t="s" s="7">
         <v>965</v>
       </c>
-      <c r="H17" t="s" s="7">
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" t="s" s="7">
+        <v>963</v>
+      </c>
+      <c r="K17" t="s" s="7">
+        <v>896</v>
+      </c>
+      <c r="L17" t="s" s="7">
         <v>966</v>
       </c>
-      <c r="I17" t="s" s="7">
-        <v>897</v>
-      </c>
-      <c r="J17" s="8"/>
-      <c r="K17" s="8"/>
-      <c r="L17" s="8"/>
     </row>
     <row r="18" ht="13.65" customHeight="1">
       <c r="A18" t="s" s="7">
@@ -9351,15 +10070,17 @@
       <c r="G18" t="s" s="7">
         <v>970</v>
       </c>
-      <c r="H18" t="s" s="7">
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" t="s" s="7">
+        <v>968</v>
+      </c>
+      <c r="K18" t="s" s="7">
+        <v>896</v>
+      </c>
+      <c r="L18" t="s" s="7">
         <v>971</v>
       </c>
-      <c r="I18" t="s" s="7">
-        <v>897</v>
-      </c>
-      <c r="J18" s="8"/>
-      <c r="K18" s="8"/>
-      <c r="L18" s="8"/>
     </row>
     <row r="19" ht="13.65" customHeight="1">
       <c r="A19" t="s" s="7">
@@ -9381,15 +10102,17 @@
       <c r="G19" t="s" s="7">
         <v>975</v>
       </c>
-      <c r="H19" t="s" s="7">
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" t="s" s="7">
+        <v>973</v>
+      </c>
+      <c r="K19" t="s" s="7">
+        <v>896</v>
+      </c>
+      <c r="L19" t="s" s="7">
         <v>976</v>
       </c>
-      <c r="I19" t="s" s="7">
-        <v>897</v>
-      </c>
-      <c r="J19" s="8"/>
-      <c r="K19" s="8"/>
-      <c r="L19" s="8"/>
     </row>
     <row r="20" ht="13.65" customHeight="1">
       <c r="A20" t="s" s="7">
@@ -9411,15 +10134,17 @@
       <c r="G20" t="s" s="7">
         <v>980</v>
       </c>
-      <c r="H20" t="s" s="7">
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+      <c r="J20" t="s" s="7">
+        <v>978</v>
+      </c>
+      <c r="K20" t="s" s="7">
+        <v>926</v>
+      </c>
+      <c r="L20" t="s" s="7">
         <v>981</v>
       </c>
-      <c r="I20" t="s" s="7">
-        <v>927</v>
-      </c>
-      <c r="J20" s="8"/>
-      <c r="K20" s="8"/>
-      <c r="L20" s="8"/>
     </row>
     <row r="21" ht="13.65" customHeight="1">
       <c r="A21" t="s" s="7">
@@ -9441,15 +10166,17 @@
       <c r="G21" t="s" s="7">
         <v>985</v>
       </c>
-      <c r="H21" t="s" s="7">
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" t="s" s="7">
+        <v>983</v>
+      </c>
+      <c r="K21" t="s" s="7">
+        <v>926</v>
+      </c>
+      <c r="L21" t="s" s="7">
         <v>986</v>
       </c>
-      <c r="I21" t="s" s="7">
-        <v>927</v>
-      </c>
-      <c r="J21" s="8"/>
-      <c r="K21" s="8"/>
-      <c r="L21" s="8"/>
     </row>
     <row r="22" ht="13.65" customHeight="1">
       <c r="A22" t="s" s="7">
@@ -9471,15 +10198,17 @@
       <c r="G22" t="s" s="7">
         <v>970</v>
       </c>
-      <c r="H22" t="s" s="7">
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
+      <c r="J22" t="s" s="7">
+        <v>988</v>
+      </c>
+      <c r="K22" t="s" s="7">
+        <v>896</v>
+      </c>
+      <c r="L22" t="s" s="7">
         <v>990</v>
       </c>
-      <c r="I22" t="s" s="7">
-        <v>897</v>
-      </c>
-      <c r="J22" s="8"/>
-      <c r="K22" s="8"/>
-      <c r="L22" s="8"/>
     </row>
     <row r="23" ht="13.65" customHeight="1">
       <c r="A23" t="s" s="7">
@@ -9501,15 +10230,17 @@
       <c r="G23" t="s" s="7">
         <v>994</v>
       </c>
-      <c r="H23" t="s" s="7">
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+      <c r="J23" t="s" s="7">
+        <v>992</v>
+      </c>
+      <c r="K23" t="s" s="7">
+        <v>890</v>
+      </c>
+      <c r="L23" t="s" s="7">
         <v>995</v>
       </c>
-      <c r="I23" t="s" s="7">
-        <v>891</v>
-      </c>
-      <c r="J23" s="8"/>
-      <c r="K23" s="8"/>
-      <c r="L23" s="8"/>
     </row>
     <row r="24" ht="13.65" customHeight="1">
       <c r="A24" t="s" s="7">
@@ -9531,15 +10262,1522 @@
       <c r="G24" t="s" s="7">
         <v>895</v>
       </c>
-      <c r="H24" t="s" s="7">
+      <c r="H24" s="8"/>
+      <c r="I24" s="8"/>
+      <c r="J24" t="s" s="7">
+        <v>997</v>
+      </c>
+      <c r="K24" t="s" s="7">
+        <v>890</v>
+      </c>
+      <c r="L24" t="s" s="7">
         <v>999</v>
       </c>
-      <c r="I24" t="s" s="7">
-        <v>891</v>
-      </c>
-      <c r="J24" s="8"/>
-      <c r="K24" s="8"/>
-      <c r="L24" s="8"/>
+    </row>
+    <row r="25">
+      <c r="B25" t="s">
+        <v>886</v>
+      </c>
+      <c r="C25" t="s">
+        <v>1013</v>
+      </c>
+      <c r="D25" t="s">
+        <v>1014</v>
+      </c>
+      <c r="E25" t="s">
+        <v>886</v>
+      </c>
+      <c r="F25" t="s">
+        <v>1015</v>
+      </c>
+      <c r="G25" t="s">
+        <v>1016</v>
+      </c>
+      <c r="K25" t="s">
+        <v>1017</v>
+      </c>
+      <c r="L25" t="s">
+        <v>1018</v>
+      </c>
+      <c r="M25" t="s">
+        <v>1019</v>
+      </c>
+      <c r="N25" t="s">
+        <v>1018</v>
+      </c>
+      <c r="O25" t="s">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="s">
+        <v>886</v>
+      </c>
+      <c r="C26" t="s">
+        <v>1020</v>
+      </c>
+      <c r="D26" t="s">
+        <v>1021</v>
+      </c>
+      <c r="E26" t="s">
+        <v>886</v>
+      </c>
+      <c r="F26" t="s">
+        <v>1022</v>
+      </c>
+      <c r="G26" t="s">
+        <v>1023</v>
+      </c>
+      <c r="K26" t="s">
+        <v>1024</v>
+      </c>
+      <c r="L26" t="s">
+        <v>1025</v>
+      </c>
+      <c r="M26" t="s">
+        <v>1026</v>
+      </c>
+      <c r="N26" t="s">
+        <v>1025</v>
+      </c>
+      <c r="O26" t="s">
+        <v>1021</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="s">
+        <v>886</v>
+      </c>
+      <c r="C27" t="s">
+        <v>1027</v>
+      </c>
+      <c r="D27" t="s">
+        <v>1028</v>
+      </c>
+      <c r="E27" t="s">
+        <v>886</v>
+      </c>
+      <c r="F27" t="s">
+        <v>1029</v>
+      </c>
+      <c r="G27" t="s">
+        <v>1030</v>
+      </c>
+      <c r="K27" t="s">
+        <v>1031</v>
+      </c>
+      <c r="L27" t="s">
+        <v>1032</v>
+      </c>
+      <c r="M27" t="s">
+        <v>1033</v>
+      </c>
+      <c r="N27" t="s">
+        <v>1032</v>
+      </c>
+      <c r="O27" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="s">
+        <v>886</v>
+      </c>
+      <c r="C28" t="s">
+        <v>1034</v>
+      </c>
+      <c r="D28" t="s">
+        <v>1035</v>
+      </c>
+      <c r="E28" t="s">
+        <v>886</v>
+      </c>
+      <c r="F28" t="s">
+        <v>1036</v>
+      </c>
+      <c r="G28" t="s">
+        <v>1037</v>
+      </c>
+      <c r="K28" t="s">
+        <v>1024</v>
+      </c>
+      <c r="L28" t="s">
+        <v>1038</v>
+      </c>
+      <c r="M28" t="s">
+        <v>1039</v>
+      </c>
+      <c r="N28" t="s">
+        <v>1038</v>
+      </c>
+      <c r="O28" t="s">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="s">
+        <v>886</v>
+      </c>
+      <c r="C29" t="s">
+        <v>1040</v>
+      </c>
+      <c r="D29" t="s">
+        <v>1041</v>
+      </c>
+      <c r="E29" t="s">
+        <v>886</v>
+      </c>
+      <c r="F29" t="s">
+        <v>1042</v>
+      </c>
+      <c r="G29" t="s">
+        <v>1043</v>
+      </c>
+      <c r="K29" t="s">
+        <v>896</v>
+      </c>
+      <c r="L29" t="s">
+        <v>1044</v>
+      </c>
+      <c r="M29" t="s">
+        <v>1045</v>
+      </c>
+      <c r="N29" t="s">
+        <v>1044</v>
+      </c>
+      <c r="O29" t="s">
+        <v>1041</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="s">
+        <v>886</v>
+      </c>
+      <c r="C30" t="s">
+        <v>1046</v>
+      </c>
+      <c r="D30" t="s">
+        <v>1047</v>
+      </c>
+      <c r="E30" t="s">
+        <v>886</v>
+      </c>
+      <c r="F30" t="s">
+        <v>1042</v>
+      </c>
+      <c r="G30" t="s">
+        <v>1048</v>
+      </c>
+      <c r="K30" t="s">
+        <v>1049</v>
+      </c>
+      <c r="L30" t="s">
+        <v>1050</v>
+      </c>
+      <c r="M30" t="s">
+        <v>1051</v>
+      </c>
+      <c r="N30" t="s">
+        <v>1050</v>
+      </c>
+      <c r="O30" t="s">
+        <v>1047</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="s">
+        <v>886</v>
+      </c>
+      <c r="C31" t="s">
+        <v>1052</v>
+      </c>
+      <c r="D31" t="s">
+        <v>1053</v>
+      </c>
+      <c r="E31" t="s">
+        <v>886</v>
+      </c>
+      <c r="F31" t="s">
+        <v>1042</v>
+      </c>
+      <c r="G31" t="s">
+        <v>1054</v>
+      </c>
+      <c r="K31" t="s">
+        <v>1024</v>
+      </c>
+      <c r="L31" t="s">
+        <v>1055</v>
+      </c>
+      <c r="M31" t="s">
+        <v>1056</v>
+      </c>
+      <c r="N31" t="s">
+        <v>1055</v>
+      </c>
+      <c r="O31" t="s">
+        <v>1053</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="s">
+        <v>886</v>
+      </c>
+      <c r="C32" t="s">
+        <v>1057</v>
+      </c>
+      <c r="D32" t="s">
+        <v>1058</v>
+      </c>
+      <c r="E32" t="s">
+        <v>886</v>
+      </c>
+      <c r="F32" t="s">
+        <v>1059</v>
+      </c>
+      <c r="G32" t="s">
+        <v>970</v>
+      </c>
+      <c r="K32" t="s">
+        <v>1060</v>
+      </c>
+      <c r="L32" t="s">
+        <v>1061</v>
+      </c>
+      <c r="M32" t="s">
+        <v>1062</v>
+      </c>
+      <c r="N32" t="s">
+        <v>1061</v>
+      </c>
+      <c r="O32" t="s">
+        <v>1058</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="s">
+        <v>886</v>
+      </c>
+      <c r="C33" t="s">
+        <v>1063</v>
+      </c>
+      <c r="D33" t="s">
+        <v>1064</v>
+      </c>
+      <c r="E33" t="s">
+        <v>886</v>
+      </c>
+      <c r="F33" t="s">
+        <v>1065</v>
+      </c>
+      <c r="G33" t="s">
+        <v>1037</v>
+      </c>
+      <c r="K33" t="s">
+        <v>1024</v>
+      </c>
+      <c r="L33" t="s">
+        <v>1066</v>
+      </c>
+      <c r="M33" t="s">
+        <v>1067</v>
+      </c>
+      <c r="N33" t="s">
+        <v>1066</v>
+      </c>
+      <c r="O33" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="s">
+        <v>886</v>
+      </c>
+      <c r="C34" t="s">
+        <v>1068</v>
+      </c>
+      <c r="D34" t="s">
+        <v>1069</v>
+      </c>
+      <c r="E34" t="s">
+        <v>886</v>
+      </c>
+      <c r="F34" t="s">
+        <v>1070</v>
+      </c>
+      <c r="G34" t="s">
+        <v>960</v>
+      </c>
+      <c r="K34" t="s">
+        <v>926</v>
+      </c>
+      <c r="L34" t="s">
+        <v>1071</v>
+      </c>
+      <c r="M34" t="s">
+        <v>1072</v>
+      </c>
+      <c r="N34" t="s">
+        <v>1071</v>
+      </c>
+      <c r="O34" t="s">
+        <v>1069</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="s">
+        <v>886</v>
+      </c>
+      <c r="C35" t="s">
+        <v>1073</v>
+      </c>
+      <c r="D35" t="s">
+        <v>1074</v>
+      </c>
+      <c r="E35" t="s">
+        <v>886</v>
+      </c>
+      <c r="F35" t="s">
+        <v>1075</v>
+      </c>
+      <c r="G35" t="s">
+        <v>1076</v>
+      </c>
+      <c r="K35" t="s">
+        <v>1024</v>
+      </c>
+      <c r="L35" t="s">
+        <v>1077</v>
+      </c>
+      <c r="M35" t="s">
+        <v>1078</v>
+      </c>
+      <c r="N35" t="s">
+        <v>1077</v>
+      </c>
+      <c r="O35" t="s">
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" t="s">
+        <v>886</v>
+      </c>
+      <c r="C36" t="s">
+        <v>1079</v>
+      </c>
+      <c r="D36" t="s">
+        <v>1080</v>
+      </c>
+      <c r="E36" t="s">
+        <v>886</v>
+      </c>
+      <c r="F36" t="s">
+        <v>1081</v>
+      </c>
+      <c r="G36" t="s">
+        <v>1082</v>
+      </c>
+      <c r="K36" t="s">
+        <v>1083</v>
+      </c>
+      <c r="L36" t="s">
+        <v>1084</v>
+      </c>
+      <c r="M36" t="s">
+        <v>1085</v>
+      </c>
+      <c r="N36" t="s">
+        <v>1084</v>
+      </c>
+      <c r="O36" t="s">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="s">
+        <v>886</v>
+      </c>
+      <c r="C37" t="s">
+        <v>1086</v>
+      </c>
+      <c r="D37" t="s">
+        <v>1087</v>
+      </c>
+      <c r="E37" t="s">
+        <v>886</v>
+      </c>
+      <c r="F37" t="s">
+        <v>1088</v>
+      </c>
+      <c r="G37" t="s">
+        <v>1089</v>
+      </c>
+      <c r="K37" t="s">
+        <v>1024</v>
+      </c>
+      <c r="L37" t="s">
+        <v>1090</v>
+      </c>
+      <c r="M37" t="s">
+        <v>1091</v>
+      </c>
+      <c r="N37" t="s">
+        <v>1090</v>
+      </c>
+      <c r="O37" t="s">
+        <v>1087</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="s">
+        <v>886</v>
+      </c>
+      <c r="C38" t="s">
+        <v>904</v>
+      </c>
+      <c r="D38" t="s">
+        <v>1092</v>
+      </c>
+      <c r="E38" t="s">
+        <v>886</v>
+      </c>
+      <c r="F38" t="s">
+        <v>900</v>
+      </c>
+      <c r="G38" t="s">
+        <v>905</v>
+      </c>
+      <c r="K38" t="s">
+        <v>896</v>
+      </c>
+      <c r="L38" t="s">
+        <v>1093</v>
+      </c>
+      <c r="M38" t="s">
+        <v>1094</v>
+      </c>
+      <c r="N38" t="s">
+        <v>1093</v>
+      </c>
+      <c r="O38" t="s">
+        <v>1092</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="s">
+        <v>886</v>
+      </c>
+      <c r="C39" t="s">
+        <v>1095</v>
+      </c>
+      <c r="D39" t="s">
+        <v>1096</v>
+      </c>
+      <c r="E39" t="s">
+        <v>886</v>
+      </c>
+      <c r="F39" t="s">
+        <v>900</v>
+      </c>
+      <c r="G39" t="s">
+        <v>1097</v>
+      </c>
+      <c r="K39" t="s">
+        <v>1024</v>
+      </c>
+      <c r="L39" t="s">
+        <v>1098</v>
+      </c>
+      <c r="M39" t="s">
+        <v>1099</v>
+      </c>
+      <c r="N39" t="s">
+        <v>1098</v>
+      </c>
+      <c r="O39" t="s">
+        <v>1096</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="s">
+        <v>886</v>
+      </c>
+      <c r="C40" t="s">
+        <v>899</v>
+      </c>
+      <c r="D40" t="s">
+        <v>1100</v>
+      </c>
+      <c r="E40" t="s">
+        <v>886</v>
+      </c>
+      <c r="F40" t="s">
+        <v>900</v>
+      </c>
+      <c r="G40" t="s">
+        <v>901</v>
+      </c>
+      <c r="K40" t="s">
+        <v>896</v>
+      </c>
+      <c r="L40" t="s">
+        <v>1101</v>
+      </c>
+      <c r="M40" t="s">
+        <v>1102</v>
+      </c>
+      <c r="N40" t="s">
+        <v>1101</v>
+      </c>
+      <c r="O40" t="s">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="s">
+        <v>886</v>
+      </c>
+      <c r="C41" t="s">
+        <v>1103</v>
+      </c>
+      <c r="D41" t="s">
+        <v>1104</v>
+      </c>
+      <c r="E41" t="s">
+        <v>886</v>
+      </c>
+      <c r="F41" t="s">
+        <v>1105</v>
+      </c>
+      <c r="G41" t="s">
+        <v>1106</v>
+      </c>
+      <c r="K41" t="s">
+        <v>1107</v>
+      </c>
+      <c r="L41" t="s">
+        <v>1108</v>
+      </c>
+      <c r="M41" t="s">
+        <v>1109</v>
+      </c>
+      <c r="N41" t="s">
+        <v>1108</v>
+      </c>
+      <c r="O41" t="s">
+        <v>1104</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" t="s">
+        <v>886</v>
+      </c>
+      <c r="C42" t="s">
+        <v>1110</v>
+      </c>
+      <c r="D42" t="s">
+        <v>1111</v>
+      </c>
+      <c r="E42" t="s">
+        <v>886</v>
+      </c>
+      <c r="F42" t="s">
+        <v>1105</v>
+      </c>
+      <c r="G42" t="s">
+        <v>931</v>
+      </c>
+      <c r="K42" t="s">
+        <v>926</v>
+      </c>
+      <c r="L42" t="s">
+        <v>1112</v>
+      </c>
+      <c r="M42" t="s">
+        <v>1113</v>
+      </c>
+      <c r="N42" t="s">
+        <v>1112</v>
+      </c>
+      <c r="O42" t="s">
+        <v>1111</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="s">
+        <v>886</v>
+      </c>
+      <c r="C43" t="s">
+        <v>1114</v>
+      </c>
+      <c r="D43" t="s">
+        <v>1115</v>
+      </c>
+      <c r="E43" t="s">
+        <v>886</v>
+      </c>
+      <c r="F43" t="s">
+        <v>1105</v>
+      </c>
+      <c r="G43" t="s">
+        <v>1116</v>
+      </c>
+      <c r="K43" t="s">
+        <v>1117</v>
+      </c>
+      <c r="L43" t="s">
+        <v>1118</v>
+      </c>
+      <c r="M43" t="s">
+        <v>1119</v>
+      </c>
+      <c r="N43" t="s">
+        <v>1118</v>
+      </c>
+      <c r="O43" t="s">
+        <v>1115</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="s">
+        <v>886</v>
+      </c>
+      <c r="C44" t="s">
+        <v>1120</v>
+      </c>
+      <c r="D44" t="s">
+        <v>1121</v>
+      </c>
+      <c r="E44" t="s">
+        <v>886</v>
+      </c>
+      <c r="F44" t="s">
+        <v>1105</v>
+      </c>
+      <c r="G44" t="s">
+        <v>1122</v>
+      </c>
+      <c r="K44" t="s">
+        <v>1123</v>
+      </c>
+      <c r="L44" t="s">
+        <v>1124</v>
+      </c>
+      <c r="M44" t="s">
+        <v>1125</v>
+      </c>
+      <c r="N44" t="s">
+        <v>1124</v>
+      </c>
+      <c r="O44" t="s">
+        <v>1121</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="s">
+        <v>886</v>
+      </c>
+      <c r="C45" t="s">
+        <v>1126</v>
+      </c>
+      <c r="D45" t="s">
+        <v>1127</v>
+      </c>
+      <c r="E45" t="s">
+        <v>886</v>
+      </c>
+      <c r="F45" t="s">
+        <v>1128</v>
+      </c>
+      <c r="G45" t="s">
+        <v>1129</v>
+      </c>
+      <c r="K45" t="s">
+        <v>1024</v>
+      </c>
+      <c r="L45" t="s">
+        <v>1130</v>
+      </c>
+      <c r="M45" t="s">
+        <v>1131</v>
+      </c>
+      <c r="N45" t="s">
+        <v>1130</v>
+      </c>
+      <c r="O45" t="s">
+        <v>1127</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="s">
+        <v>886</v>
+      </c>
+      <c r="C46" t="s">
+        <v>1132</v>
+      </c>
+      <c r="D46" t="s">
+        <v>1133</v>
+      </c>
+      <c r="E46" t="s">
+        <v>886</v>
+      </c>
+      <c r="F46" t="s">
+        <v>1134</v>
+      </c>
+      <c r="G46" t="s">
+        <v>1135</v>
+      </c>
+      <c r="K46" t="s">
+        <v>1123</v>
+      </c>
+      <c r="L46" t="s">
+        <v>1136</v>
+      </c>
+      <c r="M46" t="s">
+        <v>1137</v>
+      </c>
+      <c r="N46" t="s">
+        <v>1136</v>
+      </c>
+      <c r="O46" t="s">
+        <v>1133</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" t="s">
+        <v>886</v>
+      </c>
+      <c r="C47" t="s">
+        <v>1138</v>
+      </c>
+      <c r="D47" t="s">
+        <v>1139</v>
+      </c>
+      <c r="E47" t="s">
+        <v>886</v>
+      </c>
+      <c r="F47" t="s">
+        <v>1140</v>
+      </c>
+      <c r="G47" t="s">
+        <v>1141</v>
+      </c>
+      <c r="K47" t="s">
+        <v>1142</v>
+      </c>
+      <c r="L47" t="s">
+        <v>1143</v>
+      </c>
+      <c r="M47" t="s">
+        <v>1144</v>
+      </c>
+      <c r="N47" t="s">
+        <v>1143</v>
+      </c>
+      <c r="O47" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="s">
+        <v>886</v>
+      </c>
+      <c r="C48" t="s">
+        <v>1145</v>
+      </c>
+      <c r="D48" t="s">
+        <v>1146</v>
+      </c>
+      <c r="E48" t="s">
+        <v>886</v>
+      </c>
+      <c r="F48" t="s">
+        <v>1147</v>
+      </c>
+      <c r="G48" t="s">
+        <v>1148</v>
+      </c>
+      <c r="K48" t="s">
+        <v>1083</v>
+      </c>
+      <c r="L48" t="s">
+        <v>1149</v>
+      </c>
+      <c r="M48" t="s">
+        <v>1150</v>
+      </c>
+      <c r="N48" t="s">
+        <v>1149</v>
+      </c>
+      <c r="O48" t="s">
+        <v>1146</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" t="s">
+        <v>886</v>
+      </c>
+      <c r="C49" t="s">
+        <v>1151</v>
+      </c>
+      <c r="D49" t="s">
+        <v>1152</v>
+      </c>
+      <c r="E49" t="s">
+        <v>886</v>
+      </c>
+      <c r="F49" t="s">
+        <v>1153</v>
+      </c>
+      <c r="G49" t="s">
+        <v>1154</v>
+      </c>
+      <c r="K49" t="s">
+        <v>1060</v>
+      </c>
+      <c r="L49" t="s">
+        <v>1155</v>
+      </c>
+      <c r="M49" t="s">
+        <v>1156</v>
+      </c>
+      <c r="N49" t="s">
+        <v>1155</v>
+      </c>
+      <c r="O49" t="s">
+        <v>1152</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="s">
+        <v>886</v>
+      </c>
+      <c r="C50" t="s">
+        <v>1157</v>
+      </c>
+      <c r="D50" t="s">
+        <v>1158</v>
+      </c>
+      <c r="E50" t="s">
+        <v>886</v>
+      </c>
+      <c r="F50" t="s">
+        <v>1159</v>
+      </c>
+      <c r="G50" t="s">
+        <v>980</v>
+      </c>
+      <c r="K50" t="s">
+        <v>926</v>
+      </c>
+      <c r="L50" t="s">
+        <v>1160</v>
+      </c>
+      <c r="M50" t="s">
+        <v>1161</v>
+      </c>
+      <c r="N50" t="s">
+        <v>1160</v>
+      </c>
+      <c r="O50" t="s">
+        <v>1158</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" t="s">
+        <v>886</v>
+      </c>
+      <c r="C51" t="s">
+        <v>1162</v>
+      </c>
+      <c r="D51" t="s">
+        <v>1163</v>
+      </c>
+      <c r="E51" t="s">
+        <v>886</v>
+      </c>
+      <c r="F51" t="s">
+        <v>894</v>
+      </c>
+      <c r="G51" t="s">
+        <v>1164</v>
+      </c>
+      <c r="K51" t="s">
+        <v>1117</v>
+      </c>
+      <c r="L51" t="s">
+        <v>1165</v>
+      </c>
+      <c r="M51" t="s">
+        <v>1166</v>
+      </c>
+      <c r="N51" t="s">
+        <v>1165</v>
+      </c>
+      <c r="O51" t="s">
+        <v>1163</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="s">
+        <v>886</v>
+      </c>
+      <c r="C52" t="s">
+        <v>893</v>
+      </c>
+      <c r="D52" t="s">
+        <v>1167</v>
+      </c>
+      <c r="E52" t="s">
+        <v>886</v>
+      </c>
+      <c r="F52" t="s">
+        <v>894</v>
+      </c>
+      <c r="G52" t="s">
+        <v>895</v>
+      </c>
+      <c r="K52" t="s">
+        <v>896</v>
+      </c>
+      <c r="L52" t="s">
+        <v>1168</v>
+      </c>
+      <c r="M52" t="s">
+        <v>1169</v>
+      </c>
+      <c r="N52" t="s">
+        <v>1168</v>
+      </c>
+      <c r="O52" t="s">
+        <v>1167</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="s">
+        <v>886</v>
+      </c>
+      <c r="C53" t="s">
+        <v>988</v>
+      </c>
+      <c r="D53" t="s">
+        <v>1170</v>
+      </c>
+      <c r="E53" t="s">
+        <v>886</v>
+      </c>
+      <c r="F53" t="s">
+        <v>989</v>
+      </c>
+      <c r="G53" t="s">
+        <v>970</v>
+      </c>
+      <c r="K53" t="s">
+        <v>896</v>
+      </c>
+      <c r="L53" t="s">
+        <v>1171</v>
+      </c>
+      <c r="M53" t="s">
+        <v>1172</v>
+      </c>
+      <c r="N53" t="s">
+        <v>1171</v>
+      </c>
+      <c r="O53" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="s">
+        <v>886</v>
+      </c>
+      <c r="C54" t="s">
+        <v>1173</v>
+      </c>
+      <c r="D54" t="s">
+        <v>1174</v>
+      </c>
+      <c r="E54" t="s">
+        <v>886</v>
+      </c>
+      <c r="F54" t="s">
+        <v>1175</v>
+      </c>
+      <c r="G54" t="s">
+        <v>1054</v>
+      </c>
+      <c r="K54" t="s">
+        <v>1123</v>
+      </c>
+      <c r="L54" t="s">
+        <v>1176</v>
+      </c>
+      <c r="M54" t="s">
+        <v>1177</v>
+      </c>
+      <c r="N54" t="s">
+        <v>1176</v>
+      </c>
+      <c r="O54" t="s">
+        <v>1174</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="s">
+        <v>886</v>
+      </c>
+      <c r="C55" t="s">
+        <v>1178</v>
+      </c>
+      <c r="D55" t="s">
+        <v>1179</v>
+      </c>
+      <c r="E55" t="s">
+        <v>886</v>
+      </c>
+      <c r="F55" t="s">
+        <v>1180</v>
+      </c>
+      <c r="G55" t="s">
+        <v>985</v>
+      </c>
+      <c r="K55" t="s">
+        <v>1017</v>
+      </c>
+      <c r="L55" t="s">
+        <v>1181</v>
+      </c>
+      <c r="M55" t="s">
+        <v>1182</v>
+      </c>
+      <c r="N55" t="s">
+        <v>1181</v>
+      </c>
+      <c r="O55" t="s">
+        <v>1179</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" t="s">
+        <v>886</v>
+      </c>
+      <c r="C56" t="s">
+        <v>1183</v>
+      </c>
+      <c r="D56" t="s">
+        <v>1184</v>
+      </c>
+      <c r="E56" t="s">
+        <v>886</v>
+      </c>
+      <c r="F56" t="s">
+        <v>1185</v>
+      </c>
+      <c r="G56" t="s">
+        <v>1186</v>
+      </c>
+      <c r="K56" t="s">
+        <v>1024</v>
+      </c>
+      <c r="L56" t="s">
+        <v>1187</v>
+      </c>
+      <c r="M56" t="s">
+        <v>1188</v>
+      </c>
+      <c r="N56" t="s">
+        <v>1187</v>
+      </c>
+      <c r="O56" t="s">
+        <v>1184</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" t="s">
+        <v>886</v>
+      </c>
+      <c r="C57" t="s">
+        <v>1189</v>
+      </c>
+      <c r="D57" t="s">
+        <v>1190</v>
+      </c>
+      <c r="E57" t="s">
+        <v>886</v>
+      </c>
+      <c r="F57" t="s">
+        <v>1191</v>
+      </c>
+      <c r="G57" t="s">
+        <v>985</v>
+      </c>
+      <c r="K57" t="s">
+        <v>926</v>
+      </c>
+      <c r="L57" t="s">
+        <v>1192</v>
+      </c>
+      <c r="M57" t="s">
+        <v>1193</v>
+      </c>
+      <c r="N57" t="s">
+        <v>1192</v>
+      </c>
+      <c r="O57" t="s">
+        <v>1190</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" t="s">
+        <v>886</v>
+      </c>
+      <c r="C58" t="s">
+        <v>1194</v>
+      </c>
+      <c r="D58" t="s">
+        <v>1195</v>
+      </c>
+      <c r="E58" t="s">
+        <v>886</v>
+      </c>
+      <c r="F58" t="s">
+        <v>1196</v>
+      </c>
+      <c r="G58" t="s">
+        <v>1122</v>
+      </c>
+      <c r="K58" t="s">
+        <v>890</v>
+      </c>
+      <c r="L58" t="s">
+        <v>1197</v>
+      </c>
+      <c r="M58" t="s">
+        <v>1198</v>
+      </c>
+      <c r="N58" t="s">
+        <v>1197</v>
+      </c>
+      <c r="O58" t="s">
+        <v>1195</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" t="s">
+        <v>886</v>
+      </c>
+      <c r="C59" t="s">
+        <v>1199</v>
+      </c>
+      <c r="D59" t="s">
+        <v>1200</v>
+      </c>
+      <c r="E59" t="s">
+        <v>886</v>
+      </c>
+      <c r="F59" t="s">
+        <v>1201</v>
+      </c>
+      <c r="G59" t="s">
+        <v>910</v>
+      </c>
+      <c r="K59" t="s">
+        <v>896</v>
+      </c>
+      <c r="L59" t="s">
+        <v>1202</v>
+      </c>
+      <c r="M59" t="s">
+        <v>1203</v>
+      </c>
+      <c r="N59" t="s">
+        <v>1202</v>
+      </c>
+      <c r="O59" t="s">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" t="s">
+        <v>886</v>
+      </c>
+      <c r="C60" t="s">
+        <v>1204</v>
+      </c>
+      <c r="D60" t="s">
+        <v>1205</v>
+      </c>
+      <c r="E60" t="s">
+        <v>886</v>
+      </c>
+      <c r="F60" t="s">
+        <v>888</v>
+      </c>
+      <c r="G60" t="s">
+        <v>1089</v>
+      </c>
+      <c r="K60" t="s">
+        <v>1107</v>
+      </c>
+      <c r="L60" t="s">
+        <v>1206</v>
+      </c>
+      <c r="M60" t="s">
+        <v>1207</v>
+      </c>
+      <c r="N60" t="s">
+        <v>1206</v>
+      </c>
+      <c r="O60" t="s">
+        <v>1205</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" t="s">
+        <v>886</v>
+      </c>
+      <c r="C61" t="s">
+        <v>1208</v>
+      </c>
+      <c r="D61" t="s">
+        <v>1209</v>
+      </c>
+      <c r="E61" t="s">
+        <v>886</v>
+      </c>
+      <c r="F61" t="s">
+        <v>888</v>
+      </c>
+      <c r="G61" t="s">
+        <v>1016</v>
+      </c>
+      <c r="K61" t="s">
+        <v>1060</v>
+      </c>
+      <c r="L61" t="s">
+        <v>1210</v>
+      </c>
+      <c r="M61" t="s">
+        <v>1211</v>
+      </c>
+      <c r="N61" t="s">
+        <v>1210</v>
+      </c>
+      <c r="O61" t="s">
+        <v>1209</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" t="s">
+        <v>886</v>
+      </c>
+      <c r="C62" t="s">
+        <v>887</v>
+      </c>
+      <c r="D62" t="s">
+        <v>1212</v>
+      </c>
+      <c r="E62" t="s">
+        <v>886</v>
+      </c>
+      <c r="F62" t="s">
+        <v>888</v>
+      </c>
+      <c r="G62" t="s">
+        <v>889</v>
+      </c>
+      <c r="K62" t="s">
+        <v>890</v>
+      </c>
+      <c r="L62" t="s">
+        <v>1213</v>
+      </c>
+      <c r="M62" t="s">
+        <v>1214</v>
+      </c>
+      <c r="N62" t="s">
+        <v>1213</v>
+      </c>
+      <c r="O62" t="s">
+        <v>1212</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="s">
+        <v>886</v>
+      </c>
+      <c r="C63" t="s">
+        <v>1215</v>
+      </c>
+      <c r="D63" t="s">
+        <v>1216</v>
+      </c>
+      <c r="E63" t="s">
+        <v>886</v>
+      </c>
+      <c r="F63" t="s">
+        <v>1217</v>
+      </c>
+      <c r="G63" t="s">
+        <v>1218</v>
+      </c>
+      <c r="K63" t="s">
+        <v>1117</v>
+      </c>
+      <c r="L63" t="s">
+        <v>1219</v>
+      </c>
+      <c r="M63" t="s">
+        <v>1220</v>
+      </c>
+      <c r="N63" t="s">
+        <v>1219</v>
+      </c>
+      <c r="O63" t="s">
+        <v>1216</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" t="s">
+        <v>886</v>
+      </c>
+      <c r="C64" t="s">
+        <v>1221</v>
+      </c>
+      <c r="D64" t="s">
+        <v>1222</v>
+      </c>
+      <c r="E64" t="s">
+        <v>886</v>
+      </c>
+      <c r="F64" t="s">
+        <v>1217</v>
+      </c>
+      <c r="G64" t="s">
+        <v>955</v>
+      </c>
+      <c r="K64" t="s">
+        <v>926</v>
+      </c>
+      <c r="L64" t="s">
+        <v>1223</v>
+      </c>
+      <c r="M64" t="s">
+        <v>1224</v>
+      </c>
+      <c r="N64" t="s">
+        <v>1223</v>
+      </c>
+      <c r="O64" t="s">
+        <v>1222</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" t="s">
+        <v>886</v>
+      </c>
+      <c r="C65" t="s">
+        <v>923</v>
+      </c>
+      <c r="D65" t="s">
+        <v>1225</v>
+      </c>
+      <c r="E65" t="s">
+        <v>886</v>
+      </c>
+      <c r="F65" t="s">
+        <v>924</v>
+      </c>
+      <c r="G65" t="s">
+        <v>925</v>
+      </c>
+      <c r="K65" t="s">
+        <v>926</v>
+      </c>
+      <c r="L65" t="s">
+        <v>1226</v>
+      </c>
+      <c r="M65" t="s">
+        <v>1227</v>
+      </c>
+      <c r="N65" t="s">
+        <v>1226</v>
+      </c>
+      <c r="O65" t="s">
+        <v>1225</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="s">
+        <v>886</v>
+      </c>
+      <c r="C66" t="s">
+        <v>1228</v>
+      </c>
+      <c r="D66" t="s">
+        <v>1229</v>
+      </c>
+      <c r="E66" t="s">
+        <v>886</v>
+      </c>
+      <c r="F66" t="s">
+        <v>1230</v>
+      </c>
+      <c r="G66" t="s">
+        <v>895</v>
+      </c>
+      <c r="K66" t="s">
+        <v>890</v>
+      </c>
+      <c r="L66" t="s">
+        <v>1231</v>
+      </c>
+      <c r="M66" t="s">
+        <v>1232</v>
+      </c>
+      <c r="N66" t="s">
+        <v>1231</v>
+      </c>
+      <c r="O66" t="s">
+        <v>1229</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" t="s">
+        <v>886</v>
+      </c>
+      <c r="C67" t="s">
+        <v>918</v>
+      </c>
+      <c r="D67" t="s">
+        <v>1233</v>
+      </c>
+      <c r="E67" t="s">
+        <v>886</v>
+      </c>
+      <c r="F67" t="s">
+        <v>919</v>
+      </c>
+      <c r="G67" t="s">
+        <v>920</v>
+      </c>
+      <c r="K67" t="s">
+        <v>896</v>
+      </c>
+      <c r="L67" t="s">
+        <v>1234</v>
+      </c>
+      <c r="M67" t="s">
+        <v>1235</v>
+      </c>
+      <c r="N67" t="s">
+        <v>1234</v>
+      </c>
+      <c r="O67" t="s">
+        <v>1233</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811" footer="0.511811"/>

</xml_diff>